<commit_message>
Removendo planilhas do rastreamento para focar apenas no código
</commit_message>
<xml_diff>
--- a/ARQUIVOS_GERADOS/BI_ABASTECIMENTO/OS_FIM.xlsx
+++ b/ARQUIVOS_GERADOS/BI_ABASTECIMENTO/OS_FIM.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -649,16 +649,16 @@
         <v>180121</v>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -845,7 +845,7 @@
         <v>85</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">
@@ -856,7 +856,7 @@
         <v>36723</v>
       </c>
       <c r="C19" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -865,10 +865,10 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20">
@@ -902,7 +902,7 @@
         <v>100080</v>
       </c>
       <c r="C21" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
@@ -911,10 +911,10 @@
         <v>13</v>
       </c>
       <c r="F21" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -960,7 +960,7 @@
         <v>102</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24">
@@ -971,16 +971,16 @@
         <v>122114</v>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>105</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -994,16 +994,16 @@
         <v>122268</v>
       </c>
       <c r="C25" t="n">
-        <v>161</v>
+        <v>197</v>
       </c>
       <c r="D25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E25" t="n">
         <v>67</v>
       </c>
       <c r="F25" t="n">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1014,22 +1014,22 @@
         <v>46133</v>
       </c>
       <c r="B26" t="n">
-        <v>122591</v>
+        <v>122586</v>
       </c>
       <c r="C26" t="n">
+        <v>90</v>
+      </c>
+      <c r="D26" t="n">
         <v>4</v>
       </c>
-      <c r="D26" t="n">
-        <v>2</v>
-      </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -1037,19 +1037,19 @@
         <v>46133</v>
       </c>
       <c r="B27" t="n">
-        <v>122592</v>
+        <v>122591</v>
       </c>
       <c r="C27" t="n">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>120</v>
+        <v>41</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1060,22 +1060,22 @@
         <v>46133</v>
       </c>
       <c r="B28" t="n">
-        <v>122626</v>
+        <v>122592</v>
       </c>
       <c r="C28" t="n">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29">
@@ -1083,22 +1083,22 @@
         <v>46133</v>
       </c>
       <c r="B29" t="n">
-        <v>180033</v>
+        <v>122621</v>
       </c>
       <c r="C29" t="n">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1106,22 +1106,22 @@
         <v>46133</v>
       </c>
       <c r="B30" t="n">
-        <v>180110</v>
+        <v>122626</v>
       </c>
       <c r="C30" t="n">
         <v>75</v>
       </c>
       <c r="D30" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -1129,22 +1129,22 @@
         <v>46133</v>
       </c>
       <c r="B31" t="n">
-        <v>180121</v>
+        <v>180033</v>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>75</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32">
@@ -1152,16 +1152,16 @@
         <v>46133</v>
       </c>
       <c r="B32" t="n">
-        <v>180143</v>
+        <v>180110</v>
       </c>
       <c r="C32" t="n">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D32" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="E32" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F32" t="n">
         <v>2</v>
@@ -1175,19 +1175,19 @@
         <v>46133</v>
       </c>
       <c r="B33" t="n">
-        <v>180221</v>
+        <v>180121</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -1198,19 +1198,19 @@
         <v>46133</v>
       </c>
       <c r="B34" t="n">
-        <v>180698</v>
+        <v>180143</v>
       </c>
       <c r="C34" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="D34" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E34" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F34" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1221,19 +1221,19 @@
         <v>46133</v>
       </c>
       <c r="B35" t="n">
-        <v>180775</v>
+        <v>180221</v>
       </c>
       <c r="C35" t="n">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1244,22 +1244,22 @@
         <v>46133</v>
       </c>
       <c r="B36" t="n">
-        <v>180782</v>
+        <v>180698</v>
       </c>
       <c r="C36" t="n">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E36" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37">
@@ -1267,19 +1267,19 @@
         <v>46133</v>
       </c>
       <c r="B37" t="n">
-        <v>180794</v>
+        <v>180774</v>
       </c>
       <c r="C37" t="n">
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -1290,22 +1290,22 @@
         <v>46133</v>
       </c>
       <c r="B38" t="n">
-        <v>180889</v>
+        <v>180775</v>
       </c>
       <c r="C38" t="n">
-        <v>58</v>
+        <v>199</v>
       </c>
       <c r="D38" t="n">
-        <v>16</v>
+        <v>81</v>
       </c>
       <c r="E38" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>4</v>
+        <v>118</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -1313,19 +1313,19 @@
         <v>46133</v>
       </c>
       <c r="B39" t="n">
-        <v>180906</v>
+        <v>180782</v>
       </c>
       <c r="C39" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -1336,16 +1336,16 @@
         <v>46133</v>
       </c>
       <c r="B40" t="n">
-        <v>180917</v>
+        <v>180794</v>
       </c>
       <c r="C40" t="n">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="D40" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E40" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="F40" t="n">
         <v>6</v>
@@ -1359,22 +1359,22 @@
         <v>46133</v>
       </c>
       <c r="B41" t="n">
-        <v>180919</v>
+        <v>180889</v>
       </c>
       <c r="C41" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="D41" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E41" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="F41" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1382,22 +1382,22 @@
         <v>46133</v>
       </c>
       <c r="B42" t="n">
-        <v>180920</v>
+        <v>180906</v>
       </c>
       <c r="C42" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="D42" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E42" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43">
@@ -1405,19 +1405,19 @@
         <v>46133</v>
       </c>
       <c r="B43" t="n">
-        <v>181044</v>
+        <v>180917</v>
       </c>
       <c r="C43" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D43" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E43" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F43" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -1428,22 +1428,22 @@
         <v>46133</v>
       </c>
       <c r="B44" t="n">
-        <v>181181</v>
+        <v>180919</v>
       </c>
       <c r="C44" t="n">
+        <v>71</v>
+      </c>
+      <c r="D44" t="n">
+        <v>16</v>
+      </c>
+      <c r="E44" t="n">
+        <v>46</v>
+      </c>
+      <c r="F44" t="n">
+        <v>9</v>
+      </c>
+      <c r="G44" t="n">
         <v>2</v>
-      </c>
-      <c r="D44" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1451,19 +1451,19 @@
         <v>46133</v>
       </c>
       <c r="B45" t="n">
-        <v>181273</v>
+        <v>180920</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -1474,16 +1474,16 @@
         <v>46133</v>
       </c>
       <c r="B46" t="n">
-        <v>181287</v>
+        <v>180953</v>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -1494,22 +1494,22 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="B47" t="n">
-        <v>1224</v>
+        <v>181012</v>
       </c>
       <c r="C47" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -1517,22 +1517,22 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="B48" t="n">
-        <v>36723</v>
+        <v>181044</v>
       </c>
       <c r="C48" t="n">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="F48" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -1540,22 +1540,22 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="B49" t="n">
-        <v>122268</v>
+        <v>181181</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -1563,22 +1563,22 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="B50" t="n">
-        <v>122592</v>
+        <v>181273</v>
       </c>
       <c r="C50" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -1586,22 +1586,22 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="B51" t="n">
-        <v>122626</v>
+        <v>181287</v>
       </c>
       <c r="C51" t="n">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" t="n">
         <v>3</v>
       </c>
       <c r="F51" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -1609,22 +1609,22 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="B52" t="n">
-        <v>180033</v>
+        <v>181292</v>
       </c>
       <c r="C52" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -1635,19 +1635,19 @@
         <v>46134</v>
       </c>
       <c r="B53" t="n">
-        <v>180110</v>
+        <v>1224</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>153</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>143</v>
       </c>
       <c r="G53" t="n">
         <v>0</v>
@@ -1658,13 +1658,13 @@
         <v>46134</v>
       </c>
       <c r="B54" t="n">
-        <v>180143</v>
+        <v>26082</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
@@ -1681,19 +1681,19 @@
         <v>46134</v>
       </c>
       <c r="B55" t="n">
-        <v>180774</v>
+        <v>36723</v>
       </c>
       <c r="C55" t="n">
-        <v>41</v>
+        <v>129</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>24</v>
+        <v>127</v>
       </c>
       <c r="G55" t="n">
         <v>0</v>
@@ -1704,19 +1704,19 @@
         <v>46134</v>
       </c>
       <c r="B56" t="n">
-        <v>180794</v>
+        <v>100080</v>
       </c>
       <c r="C56" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E56" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -1727,19 +1727,19 @@
         <v>46134</v>
       </c>
       <c r="B57" t="n">
-        <v>180889</v>
+        <v>100873</v>
       </c>
       <c r="C57" t="n">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E57" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -1750,19 +1750,19 @@
         <v>46134</v>
       </c>
       <c r="B58" t="n">
-        <v>180917</v>
+        <v>122114</v>
       </c>
       <c r="C58" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E58" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
@@ -1773,19 +1773,19 @@
         <v>46134</v>
       </c>
       <c r="B59" t="n">
-        <v>180919</v>
+        <v>122268</v>
       </c>
       <c r="C59" t="n">
-        <v>15</v>
+        <v>327</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="E59" t="n">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -1796,19 +1796,19 @@
         <v>46134</v>
       </c>
       <c r="B60" t="n">
-        <v>180920</v>
+        <v>122586</v>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -1819,21 +1819,619 @@
         <v>46134</v>
       </c>
       <c r="B61" t="n">
+        <v>122591</v>
+      </c>
+      <c r="C61" t="n">
+        <v>25</v>
+      </c>
+      <c r="D61" t="n">
+        <v>11</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>14</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B62" t="n">
+        <v>122592</v>
+      </c>
+      <c r="C62" t="n">
+        <v>152</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="n">
+        <v>5</v>
+      </c>
+      <c r="F62" t="n">
+        <v>146</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B63" t="n">
+        <v>122621</v>
+      </c>
+      <c r="C63" t="n">
+        <v>38</v>
+      </c>
+      <c r="D63" t="n">
+        <v>5</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>33</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B64" t="n">
+        <v>122626</v>
+      </c>
+      <c r="C64" t="n">
+        <v>110</v>
+      </c>
+      <c r="D64" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" t="n">
+        <v>104</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B65" t="n">
+        <v>122692</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B66" t="n">
+        <v>180033</v>
+      </c>
+      <c r="C66" t="n">
+        <v>87</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>87</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B67" t="n">
+        <v>180101</v>
+      </c>
+      <c r="C67" t="n">
+        <v>17</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" t="n">
+        <v>9</v>
+      </c>
+      <c r="F67" t="n">
+        <v>7</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B68" t="n">
+        <v>180110</v>
+      </c>
+      <c r="C68" t="n">
+        <v>30</v>
+      </c>
+      <c r="D68" t="n">
+        <v>28</v>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B69" t="n">
+        <v>180121</v>
+      </c>
+      <c r="C69" t="n">
+        <v>6</v>
+      </c>
+      <c r="D69" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>3</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B70" t="n">
+        <v>180143</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B71" t="n">
+        <v>180221</v>
+      </c>
+      <c r="C71" t="n">
+        <v>30</v>
+      </c>
+      <c r="D71" t="n">
+        <v>29</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B72" t="n">
+        <v>180698</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B73" t="n">
+        <v>180774</v>
+      </c>
+      <c r="C73" t="n">
+        <v>254</v>
+      </c>
+      <c r="D73" t="n">
+        <v>20</v>
+      </c>
+      <c r="E73" t="n">
+        <v>104</v>
+      </c>
+      <c r="F73" t="n">
+        <v>130</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B74" t="n">
+        <v>180775</v>
+      </c>
+      <c r="C74" t="n">
+        <v>48</v>
+      </c>
+      <c r="D74" t="n">
+        <v>19</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>29</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B75" t="n">
+        <v>180782</v>
+      </c>
+      <c r="C75" t="n">
+        <v>20</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>14</v>
+      </c>
+      <c r="F75" t="n">
+        <v>6</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B76" t="n">
+        <v>180794</v>
+      </c>
+      <c r="C76" t="n">
+        <v>156</v>
+      </c>
+      <c r="D76" t="n">
+        <v>42</v>
+      </c>
+      <c r="E76" t="n">
+        <v>100</v>
+      </c>
+      <c r="F76" t="n">
+        <v>14</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B77" t="n">
+        <v>180869</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B78" t="n">
+        <v>180889</v>
+      </c>
+      <c r="C78" t="n">
+        <v>77</v>
+      </c>
+      <c r="D78" t="n">
+        <v>39</v>
+      </c>
+      <c r="E78" t="n">
+        <v>38</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B79" t="n">
+        <v>180906</v>
+      </c>
+      <c r="C79" t="n">
+        <v>27</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>27</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B80" t="n">
+        <v>180917</v>
+      </c>
+      <c r="C80" t="n">
+        <v>94</v>
+      </c>
+      <c r="D80" t="n">
+        <v>21</v>
+      </c>
+      <c r="E80" t="n">
+        <v>65</v>
+      </c>
+      <c r="F80" t="n">
+        <v>8</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B81" t="n">
+        <v>180919</v>
+      </c>
+      <c r="C81" t="n">
+        <v>135</v>
+      </c>
+      <c r="D81" t="n">
+        <v>44</v>
+      </c>
+      <c r="E81" t="n">
+        <v>82</v>
+      </c>
+      <c r="F81" t="n">
+        <v>9</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B82" t="n">
+        <v>180920</v>
+      </c>
+      <c r="C82" t="n">
+        <v>61</v>
+      </c>
+      <c r="D82" t="n">
+        <v>28</v>
+      </c>
+      <c r="E82" t="n">
+        <v>32</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B83" t="n">
+        <v>181012</v>
+      </c>
+      <c r="C83" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B84" t="n">
         <v>181044</v>
       </c>
-      <c r="C61" t="n">
-        <v>20</v>
-      </c>
-      <c r="D61" t="n">
-        <v>4</v>
-      </c>
-      <c r="E61" t="n">
-        <v>12</v>
-      </c>
-      <c r="F61" t="n">
-        <v>4</v>
-      </c>
-      <c r="G61" t="n">
+      <c r="C84" t="n">
+        <v>109</v>
+      </c>
+      <c r="D84" t="n">
+        <v>58</v>
+      </c>
+      <c r="E84" t="n">
+        <v>41</v>
+      </c>
+      <c r="F84" t="n">
+        <v>10</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B85" t="n">
+        <v>181048</v>
+      </c>
+      <c r="C85" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B86" t="n">
+        <v>181181</v>
+      </c>
+      <c r="C86" t="n">
+        <v>17</v>
+      </c>
+      <c r="D86" t="n">
+        <v>17</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B87" t="n">
+        <v>181292</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>